<commit_message>
Add .gitattributes to stop office/image files being treated as text
The previous commit's ภารกิจ v2.xlsx got silently mangled by Git's CRLF
auto-conversion (no .gitattributes existed, so Git guessed it was text).
Mark .xlsx/.doc(x)/.pdf/image extensions as binary so this can't happen
again, and re-add the xlsx so its stored blob matches the original file
byte-for-byte.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/xlsx/ภารกิจ v2.xlsx
+++ b/docs/xlsx/ภารกิจ v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\เกมอสม\docs\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2B3B644E-F4D5-48B9-BEB2-91ECA1F8E833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D79FD976-0CD4-46E0-8735-87C8910ADE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{898338AB-F174-4A37-8858-20635A8A1EE6}"/>
   </bookViews>
@@ -2071,8 +2071,9 @@
     <col min="3" max="3" width="25.54296875" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
     <col min="5" max="5" width="62.7265625" customWidth="1"/>
-    <col min="6" max="6" width="52.81640625" customWidth="1"/>
-    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.90625" customWidth="1"/>
+    <col min="7" max="7" width="21.36328125" customWidth="1"/>
+    <col min="8" max="8" width="17.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="95.65" x14ac:dyDescent="0.45">

</xml_diff>